<commit_message>
Added Decision lab feedback
</commit_message>
<xml_diff>
--- a/public/templates/decision-lab-import-template.xlsx
+++ b/public/templates/decision-lab-import-template.xlsx
@@ -214,6 +214,11 @@
         <t>Textul de consecință afișat imediat după ce jucătorul alege această opțiune.</t>
       </text>
     </comment>
+    <comment ref="K1" authorId="0" shapeId="0">
+      <text>
+        <t>Opțional. Eticheta comportamentală a opțiunii, folosită pentru profilul final: exploration, execution, analysis, diplomacy sau investigation. Poate rămâne gol.</t>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -507,7 +512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -520,6 +525,7 @@
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="8" customWidth="1" min="9" max="9"/>
     <col width="40" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -573,6 +579,11 @@
           <t>feedback</t>
         </is>
       </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>trait</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -625,6 +636,11 @@
           <t>Clientul e mulțumit pe moment, dar ai creat un precedent riscant fără verificări.</t>
         </is>
       </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>execution</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -673,6 +689,11 @@
           <t>Ai echilibrat presiunea comercială cu prudența necesară.</t>
         </is>
       </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>exploration</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -721,6 +742,11 @@
           <t>Decizia ajunge la nivelul potrivit, dar procesul devine mai lent.</t>
         </is>
       </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>diplomacy</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -767,6 +793,11 @@
       <c r="J5" s="2" t="inlineStr">
         <is>
           <t>Ai respectat procedura, dar riști să pierzi încrederea clientului.</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>execution</t>
         </is>
       </c>
     </row>
@@ -801,6 +832,7 @@
       <c r="H6" s="2" t="inlineStr"/>
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr"/>
+      <c r="K6" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -814,7 +846,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -886,7 +918,14 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>9. Salvează și încarcă fișierul în /admin/decision-lab/, la Import.</t>
+          <t>9. Coloana 'trait' e opțională — dacă o completezi (exploration/execution/analysis/diplomacy/investigation), opțiunea contribuie la profilul final afișat jucătorului.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>10. Salvează și încarcă fișierul în /admin/decision-lab/, la Import.</t>
         </is>
       </c>
     </row>

</xml_diff>